<commit_message>
update edición masiva: aumentos, agregados, simulación por pedido y hoja Instrucciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/abastecimiento/anulador/assets/PlantillaEdicion.xlsx
+++ b/abastecimiento/anulador/assets/PlantillaEdicion.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EdicionPedidos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,4 +478,52 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="95" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>1. Una fila por artículo y pedido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2. NUEVA_CANTIDAD es la cantidad total que tiene que quedar en el pedido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3. 0 quita el artículo del pedido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4. Si el artículo no está en el pedido, se agrega con esa cantidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5. Antes de aplicar se valida el stock y, para franquicias y mayoristas, el crédito.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>